<commit_message>
Sprit magic working failry well. Clean up branches
</commit_message>
<xml_diff>
--- a/Data/Cults.xlsx
+++ b/Data/Cults.xlsx
@@ -1,21 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\Stat_blocks\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354D04BF-6E85-4C09-B5BE-D13E7648E9E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D72B8830-3DCA-4BFA-A585-69A3CDDC6356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40890" yWindow="2175" windowWidth="28800" windowHeight="15345" xr2:uid="{6FB7BD71-90B3-45D5-8369-ED5846415A0F}"/>
+    <workbookView xWindow="3240" yWindow="1245" windowWidth="32175" windowHeight="19260" activeTab="6" xr2:uid="{6FB7BD71-90B3-45D5-8369-ED5846415A0F}"/>
   </bookViews>
   <sheets>
     <sheet name="Thed_Magic" sheetId="4" r:id="rId1"/>
     <sheet name="Thed_Roles" sheetId="3" r:id="rId2"/>
     <sheet name="Thed_Associations" sheetId="2" r:id="rId3"/>
+    <sheet name="Mallia_Magic" sheetId="5" r:id="rId4"/>
+    <sheet name="Mallia_Roles" sheetId="6" r:id="rId5"/>
+    <sheet name="Mallia_Associations" sheetId="7" r:id="rId6"/>
+    <sheet name="Kyger Litor_Magic" sheetId="8" r:id="rId7"/>
+    <sheet name="Kyger Litor_Roles" sheetId="9" r:id="rId8"/>
+    <sheet name="Kyger Litor_Associations" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="152">
   <si>
     <t>Access to Chaos Feature ritual via Primal Chaos.</t>
   </si>
@@ -299,14 +305,217 @@
   </si>
   <si>
     <t>16-22</t>
+  </si>
+  <si>
+    <t>Summons a disease spirit.</t>
+  </si>
+  <si>
+    <t>Summon Disease Spirit</t>
+  </si>
+  <si>
+    <t>Allows control over a disease spirit.</t>
+  </si>
+  <si>
+    <t>Command Disease Spirit</t>
+  </si>
+  <si>
+    <t>Target contracts disease if POW overcome; stackable for severity.</t>
+  </si>
+  <si>
+    <t>Cause (Disease)</t>
+  </si>
+  <si>
+    <t>Ritual â€“ causes immunity and carrier state.</t>
+  </si>
+  <si>
+    <t>Carry (Disease)</t>
+  </si>
+  <si>
+    <t>All spirit magic available at full price.</t>
+  </si>
+  <si>
+    <t>Full price</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Both shaman and Rune Priest; follows normal shaman rules to attain status.</t>
+  </si>
+  <si>
+    <t>Disease Master</t>
+  </si>
+  <si>
+    <t>Acceptance is automatic upon sacrificing 1 POW to create 1 Rune point. May sacrifice MP for disease protection on holy days.</t>
+  </si>
+  <si>
+    <t>Summon Fear Spirit</t>
+  </si>
+  <si>
+    <t>Summon Darkness Elemental (all sizes)</t>
+  </si>
+  <si>
+    <t>Dismiss Darkness Elemental (all sizes)</t>
+  </si>
+  <si>
+    <t>Darksee</t>
+  </si>
+  <si>
+    <t>Counterchaos</t>
+  </si>
+  <si>
+    <t>Command Fear Spirit</t>
+  </si>
+  <si>
+    <t>Blinding</t>
+  </si>
+  <si>
+    <t>Absorption</t>
+  </si>
+  <si>
+    <t>Common Rune Magic: All.</t>
+  </si>
+  <si>
+    <t>Initiates are forbidden from fire/light spells.</t>
+  </si>
+  <si>
+    <t>Prohibited</t>
+  </si>
+  <si>
+    <t>Lightwall</t>
+  </si>
+  <si>
+    <t>Light</t>
+  </si>
+  <si>
+    <t>Ignite</t>
+  </si>
+  <si>
+    <t>Fireblade</t>
+  </si>
+  <si>
+    <t>Firearrow</t>
+  </si>
+  <si>
+    <t>May be learned but should only be used against nonâ€‘trolls or in ambient light.</t>
+  </si>
+  <si>
+    <t>Allowed</t>
+  </si>
+  <si>
+    <t>Detect (substance)</t>
+  </si>
+  <si>
+    <t>Detect Magic</t>
+  </si>
+  <si>
+    <t>Available to Kyger Litor trolls.</t>
+  </si>
+  <si>
+    <t>Spirit Screen</t>
+  </si>
+  <si>
+    <t>Slow</t>
+  </si>
+  <si>
+    <t>Second Sight</t>
+  </si>
+  <si>
+    <t>Protection</t>
+  </si>
+  <si>
+    <t>Heal</t>
+  </si>
+  <si>
+    <t>Extinguish</t>
+  </si>
+  <si>
+    <t>Dullblade</t>
+  </si>
+  <si>
+    <t>Disruption</t>
+  </si>
+  <si>
+    <t>Demoralize</t>
+  </si>
+  <si>
+    <t>Darkwall</t>
+  </si>
+  <si>
+    <t>Countermagic</t>
+  </si>
+  <si>
+    <t>Bludgeon</t>
+  </si>
+  <si>
+    <t>Befuddle</t>
+  </si>
+  <si>
+    <t>Requirements: Meet Priestess reqs; then follow shaman rules and awaken fetch. Special: may only bind Darkness spirits to fetch.</t>
+  </si>
+  <si>
+    <t>Priestess-Shaman</t>
+  </si>
+  <si>
+    <t>Requirements: Standard; must have Read/Write Darktongue 30% and know Darkwall.</t>
+  </si>
+  <si>
+    <t>Priestess</t>
+  </si>
+  <si>
+    <t>Requirements: CHA 18+, Read/Write Darktongue 30%; 90% in two weapon skills and two of: Battle, Climb, Conceal, Listen, Darksense Scan, Darksense Search; pass POWÃ—3. Special: DI checks use 1D10; donate 90% time/income to cult.</t>
+  </si>
+  <si>
+    <t>Karrgs Son (Rune Lord)</t>
+  </si>
+  <si>
+    <t>Full trolls (Mistress Race, dark, great, jungle, snow) auto-initiate upon sacrificing 1 POW for 1 Rune point. Part-trolls (trollkin, tusk riders): POW 10+, Darktongue 50%, one weapon 40%+, pass POWÃ—5; then sacrifice 1 POW. Non-trolls: Darkness Rune 50%+, also meet part-troll reqs, pass POWÃ—3; failure = death. Cult skill bonuses: Cult Lore (Kyger Litor) +15%, Meditate +5%, Sing +10%, Speak Darktongue +15%, Spirit Combat +20%, Worship (Kyger Litor) +20%. Favored Passions: Devotion (Kyger Litor), Hate (Chaos), Loyalty (high priestess), Loyalty (temple).</t>
+  </si>
+  <si>
+    <t>Crush</t>
+  </si>
+  <si>
+    <t>Zorak Zoran</t>
+  </si>
+  <si>
+    <t>The Solace of the Deep Dark Within provides this.</t>
+  </si>
+  <si>
+    <t>Healing Trance</t>
+  </si>
+  <si>
+    <t>Xiola Umbar</t>
+  </si>
+  <si>
+    <t>The Goddess of Deep Dark Within provides this.</t>
+  </si>
+  <si>
+    <t>Attack Soul</t>
+  </si>
+  <si>
+    <t>Subere</t>
+  </si>
+  <si>
+    <t>Summon Specific Ancestor</t>
+  </si>
+  <si>
+    <t>Daka Fal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -334,9 +543,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -675,6 +885,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="20.85546875" customWidth="1"/>
+    <col min="5" max="5" width="33.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="69.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1248,4 +1459,826 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA985CBA-52BA-4A53-90D0-A492ED1A16E1}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FF81BBC-C4E3-42C0-94DF-157B26EED6E4}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09333154-6B5B-4443-B4CC-315083054CAF}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F336F2C0-1A11-4978-8D42-430584D99A35}">
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.5703125" customWidth="1"/>
+    <col min="4" max="4" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="72.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" t="s">
+        <v>118</v>
+      </c>
+      <c r="F3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" t="s">
+        <v>118</v>
+      </c>
+      <c r="F5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E6" t="s">
+        <v>118</v>
+      </c>
+      <c r="F6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E7" t="s">
+        <v>118</v>
+      </c>
+      <c r="F7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" t="s">
+        <v>128</v>
+      </c>
+      <c r="D8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E8" t="s">
+        <v>118</v>
+      </c>
+      <c r="F8" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" t="s">
+        <v>118</v>
+      </c>
+      <c r="F9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" t="s">
+        <v>126</v>
+      </c>
+      <c r="D10" t="s">
+        <v>70</v>
+      </c>
+      <c r="E10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" t="s">
+        <v>125</v>
+      </c>
+      <c r="D11" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" t="s">
+        <v>118</v>
+      </c>
+      <c r="F11" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" t="s">
+        <v>124</v>
+      </c>
+      <c r="D12" t="s">
+        <v>70</v>
+      </c>
+      <c r="E12" t="s">
+        <v>118</v>
+      </c>
+      <c r="F12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" t="s">
+        <v>123</v>
+      </c>
+      <c r="D13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" t="s">
+        <v>118</v>
+      </c>
+      <c r="F13" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s">
+        <v>122</v>
+      </c>
+      <c r="D14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" t="s">
+        <v>120</v>
+      </c>
+      <c r="D15" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F15" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" t="s">
+        <v>119</v>
+      </c>
+      <c r="D16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16" t="s">
+        <v>118</v>
+      </c>
+      <c r="F16" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>76</v>
+      </c>
+      <c r="B17" t="s">
+        <v>116</v>
+      </c>
+      <c r="E17" t="s">
+        <v>111</v>
+      </c>
+      <c r="F17" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" t="s">
+        <v>115</v>
+      </c>
+      <c r="E18" t="s">
+        <v>111</v>
+      </c>
+      <c r="F18" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" t="s">
+        <v>114</v>
+      </c>
+      <c r="E19" t="s">
+        <v>111</v>
+      </c>
+      <c r="F19" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" t="s">
+        <v>113</v>
+      </c>
+      <c r="E20" t="s">
+        <v>111</v>
+      </c>
+      <c r="F20" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>76</v>
+      </c>
+      <c r="B21" t="s">
+        <v>112</v>
+      </c>
+      <c r="E21" t="s">
+        <v>111</v>
+      </c>
+      <c r="F21" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" t="s">
+        <v>72</v>
+      </c>
+      <c r="E22" t="s">
+        <v>67</v>
+      </c>
+      <c r="F22" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" t="s">
+        <v>71</v>
+      </c>
+      <c r="E23" t="s">
+        <v>67</v>
+      </c>
+      <c r="F23" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" t="s">
+        <v>108</v>
+      </c>
+      <c r="D24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E24" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" t="s">
+        <v>107</v>
+      </c>
+      <c r="D25" t="s">
+        <v>58</v>
+      </c>
+      <c r="E25" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" t="s">
+        <v>106</v>
+      </c>
+      <c r="D26" t="s">
+        <v>58</v>
+      </c>
+      <c r="E26" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" t="s">
+        <v>105</v>
+      </c>
+      <c r="D27" t="s">
+        <v>58</v>
+      </c>
+      <c r="E27" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" t="s">
+        <v>104</v>
+      </c>
+      <c r="D28" t="s">
+        <v>58</v>
+      </c>
+      <c r="E28" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>56</v>
+      </c>
+      <c r="B29" t="s">
+        <v>103</v>
+      </c>
+      <c r="D29" t="s">
+        <v>58</v>
+      </c>
+      <c r="E29" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" t="s">
+        <v>102</v>
+      </c>
+      <c r="D30" t="s">
+        <v>58</v>
+      </c>
+      <c r="E30" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" t="s">
+        <v>101</v>
+      </c>
+      <c r="D31" t="s">
+        <v>58</v>
+      </c>
+      <c r="E31" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{368AE33F-606D-44D5-97AE-D01C9213EAEB}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C07F011D-6B12-49EF-BEF9-3DF64DFAC9BA}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>